<commit_message>
Revisa relatórios finais do iGovTI 2026
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/99-Avaliacao_Evidencias/painel-avaliacao-evidencias-neutro.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/99-Avaliacao_Evidencias/painel-avaliacao-evidencias-neutro.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Auditado</t>
   </si>
@@ -31,9 +31,6 @@
     <t>q0103[G]</t>
   </si>
   <si>
-    <t>q1001ext[C]</t>
-  </si>
-  <si>
     <t>q1001ext[E]</t>
   </si>
   <si>
@@ -43,21 +40,9 @@
     <t>q1001ext[H]</t>
   </si>
   <si>
-    <t>q1002ext[A]</t>
-  </si>
-  <si>
-    <t>q1002ext[C]</t>
-  </si>
-  <si>
     <t>q2101ext[A]</t>
   </si>
   <si>
-    <t>q2101ext[B]</t>
-  </si>
-  <si>
-    <t>q2101ext[C]</t>
-  </si>
-  <si>
     <t>q2101ext[D]</t>
   </si>
   <si>
@@ -91,115 +76,37 @@
     <t>q2203ext[A]</t>
   </si>
   <si>
-    <t>q2203ext[B]</t>
-  </si>
-  <si>
     <t>q2203ext[C]</t>
   </si>
   <si>
     <t>q2204ext[A]</t>
   </si>
   <si>
-    <t>q2204ext[B]</t>
-  </si>
-  <si>
-    <t>q2204ext[C]</t>
-  </si>
-  <si>
     <t>q2204ext[D]</t>
   </si>
   <si>
     <t>q2204ext[E]</t>
   </si>
   <si>
-    <t>q2204ext[F]</t>
-  </si>
-  <si>
-    <t>q2501ext[A]</t>
-  </si>
-  <si>
-    <t>q2501ext[B]</t>
-  </si>
-  <si>
     <t>q2504ext[A]</t>
   </si>
   <si>
     <t>q2504ext[B]</t>
   </si>
   <si>
-    <t>q2701ext[A]</t>
-  </si>
-  <si>
-    <t>q2701ext[C]</t>
-  </si>
-  <si>
-    <t>q2702ext[A]</t>
-  </si>
-  <si>
-    <t>q2702ext[C]</t>
-  </si>
-  <si>
-    <t>q2703ext[B]</t>
-  </si>
-  <si>
     <t>q2703ext[C]</t>
   </si>
   <si>
-    <t>q2704ext[B]</t>
-  </si>
-  <si>
-    <t>q2705ext[B]</t>
-  </si>
-  <si>
-    <t>q2705ext[C]</t>
-  </si>
-  <si>
-    <t>q2705ext[D]</t>
-  </si>
-  <si>
-    <t>q2706ext[A]</t>
-  </si>
-  <si>
-    <t>q2706ext[B]</t>
-  </si>
-  <si>
-    <t>q2706ext[C]</t>
-  </si>
-  <si>
-    <t>q2708[A]</t>
-  </si>
-  <si>
     <t>q2708[B]</t>
   </si>
   <si>
-    <t>q2708[C]</t>
-  </si>
-  <si>
     <t>q2708[D]</t>
   </si>
   <si>
     <t>q2801ext[A]</t>
   </si>
   <si>
-    <t>q2801ext[C]</t>
-  </si>
-  <si>
-    <t>q2801ext[D]</t>
-  </si>
-  <si>
-    <t>q2801ext[E]</t>
-  </si>
-  <si>
-    <t>q2801ext[F]</t>
-  </si>
-  <si>
-    <t>q2801ext[G]</t>
-  </si>
-  <si>
-    <t>q2802ext[C]</t>
-  </si>
-  <si>
-    <t>q2802ext[D]</t>
+    <t>q2801ext[B]</t>
   </si>
   <si>
     <t>q2804[A]</t>
@@ -540,10 +447,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BM1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:65">
+    <row r="1" spans="1:34">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -645,99 +552,6 @@
       </c>
       <c r="AH1" t="s">
         <v>33</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>51</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>52</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>54</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>55</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>56</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>57</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>58</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>59</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>60</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>61</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>62</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>63</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>